<commit_message>
Add Tushar Agrawal FY2026-27 YTD capital gains and dividends
Extend workbook with CG/OS sheets for 01-Apr-2026–03-Sep-2026; add
SBI TT rates through Aug-2026 for Rule 115 FX.

Co-authored-by: yashjain-a11y <yashjain-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/clients/Tushar_Agrawal_U16595399/Foreign_Assets_Schedule_FA_Tushar_Agrawal_AY2026-27.xlsx
+++ b/clients/Tushar_Agrawal_U16595399/Foreign_Assets_Schedule_FA_Tushar_Agrawal_AY2026-27.xlsx
@@ -20,6 +20,8 @@
     <sheet name="FIFO Lots Register" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="CG Summary by Symbol" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Notes for CA" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Capital Gains FY2026-27" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Schedule OS - FY2026-27" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -471,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Table range for VLOOKUP: A4:C26</t>
+          <t>Table range for VLOOKUP: A4:C33</t>
         </is>
       </c>
     </row>
@@ -859,99 +861,209 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
+      </c>
+    </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>FCY→USD cross rates (IBKR 31-Dec-2025 close — edit if using trade-date FX)</t>
+      <c r="A28" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>Units per 1 FCY → USD</t>
+      <c r="A29" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>CHF</t>
-        </is>
+      <c r="A30" s="2" t="n">
+        <v>46202</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>1.2615</v>
+        <v>93.95</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>DKK</t>
-        </is>
+      <c r="A31" s="2" t="n">
+        <v>46203</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>0.15726</v>
+        <v>93.95</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
+      <c r="A32" s="2" t="n">
+        <v>46234</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>1.1746</v>
+        <v>95.2</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>HKD</t>
-        </is>
+      <c r="A33" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>0.12849</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>0.0063827</v>
+        <v>95</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SGD</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>0.7776049766718507</v>
+          <t>FCY→USD cross rates (IBKR 31-Dec-2025 close — edit if using trade-date FX)</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37"/>
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>Units per 1 FCY → USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1.2615</v>
+      </c>
+    </row>
     <row r="38">
       <c r="A38" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0.15726</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>1.1746</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0.12849</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0.0063827</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0.7776049766718507</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Yellow/input cells on CG sheets: Sale/Cost FCY, Comm USD, FX rates. All P&amp;L columns are formulas.</t>
         </is>
@@ -1125,7 +1237,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="G6" s="4" t="n"/>
       <c r="T6" s="4" t="n"/>
@@ -1138,7 +1249,6 @@
       <c r="G8" s="4" t="n"/>
       <c r="T8" s="4" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -2442,7 +2552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2881,7 +2991,6 @@
         <v>3870.56</v>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -2892,6 +3001,331 @@
         <is>
           <t>Detail P&amp;L with editable FX is on 'Capital Gains FY2025-26' (formula-driven). This summary is a static cross-check.</t>
         </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>— FY 2026-27 YTD (to 03-Sep-2026) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>STCG INR</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>LTCG INR</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Total Gain/(Loss) INR</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sale Proceeds USD</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Cost USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1919</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>-2367</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-2367</v>
+      </c>
+      <c r="E25" t="n">
+        <v>853.17</v>
+      </c>
+      <c r="F25" t="n">
+        <v>925.9299999999999</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4568.T</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-65344</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-65344</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1626.95</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2376.26</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AAXJ</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>15367</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>15367</v>
+      </c>
+      <c r="E27" t="n">
+        <v>482.48</v>
+      </c>
+      <c r="F27" t="n">
+        <v>346.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BNO</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>25103</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>25103</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1762.53</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1507.12</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7454</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>7454</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1134.72</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1145.07</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IWR</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>9683</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>9683</v>
+      </c>
+      <c r="E30" t="n">
+        <v>540.85</v>
+      </c>
+      <c r="F30" t="n">
+        <v>474.88</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>178257</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>178257</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2451.51</v>
+      </c>
+      <c r="F31" t="n">
+        <v>614.53</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>35325</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>35325</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1435.42</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1151.67</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SLV</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>569880</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>569880</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9986.790000000001</v>
+      </c>
+      <c r="F33" t="n">
+        <v>4524.6</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TIP</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>66808</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>66808</v>
+      </c>
+      <c r="E34" t="n">
+        <v>6209.58</v>
+      </c>
+      <c r="F34" t="n">
+        <v>6185.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>URA</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>10049</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>10049</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2339.5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2374</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>27665</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>27665</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1402.56</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1203.9</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>VTV</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>19091</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>19091</v>
+      </c>
+      <c r="E37" t="n">
+        <v>872</v>
+      </c>
+      <c r="F37" t="n">
+        <v>726.38</v>
       </c>
     </row>
   </sheetData>
@@ -2905,7 +3339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2939,7 +3373,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Only FY 2025-26 Activity Statement furnished (01-Apr-2025–31-Mar-2026). 19 symbols already held at FY start (MTM Prior Qty) — opening lots seeded 31-Dec-2024 with costs backsolved from IBKR sell Basis (FIFO) or end Open Positions cost (SLV/TIP/TSLA/4568.T). True original buy dates pre-date furnished statements — confirm for LTCG clock.</t>
+          <t>FY 2025-26 Activity Statement (01-Apr-2025–31-Mar-2026) + FY 2026-27 YTD (01-Apr-2026–03-Sep-2026). 19 symbols held at FY2025-26 start — opening lots seeded 31-Dec-2024 with costs backsolved from IBKR sell Basis (FIFO) / Open Positions cost. True original buy dates pre-date furnished statements — confirm for LTCG clock.</t>
         </is>
       </c>
     </row>
@@ -2951,206 +3385,206 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Not furnished — synthesized from FY trades in CY2025 + seeds. YE2025 marks at cost. CY dividends/interest omit Jan–Mar 2025 (outside fiscal window). Prefer IBKR Annual / PortfolioAnalyst for filing.</t>
+          <t>Not furnished — synthesized from FY2025-26 trades in CY2025 + seeds. YE2025 marks at cost. CY dividends/interest omit Jan–Mar 2025. Prefer IBKR Annual / PortfolioAnalyst for filing.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Capital gains</t>
+          <t>FY 2026-27 (partial)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FY2025-26: multiple equity/ETF disposals (BLBD, AMZN, ASML, BX, CAT, GE, LLY, NFLX, TGT, TSM, XOM, NOVd, R6C0d/SHELL, ACN, CPNG, WCBR, 1810, GD, etc.). Multi-currency USD/EUR/HKD/JPY/DKK.</t>
+          <t>Sheets 'Capital Gains FY2026-27' and 'Schedule OS - FY2026-27' cover 01-Apr-2026 to 03-Sep-2026 only (statement end). Full-year FY2026-27 requires Activity Statement through 31-Mar-2027. SBI TT Apr–Aug 2026 from public TTBR compilations — verify on sbi.co.in before filing.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Peak NAV</t>
+          <t>Capital gains</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Activity Statement / synthesized peak = max(start, end) only. Obtain PortfolioAnalyst for true peak A2.</t>
+          <t>FY2025-26: BLBD/AMZN/ASML/BX/CAT/GE/LLY/NFLX/TGT/TSM/XOM/NOVd/R6C0d/ACN/CPNG/WCBR/1810/GD etc. FY2026-27 YTD: SLV/NBIS/TIP/URA/1919/4568.T/AAXJ/BNO/IEF/IWR/QQQ/VT/VTV etc.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Assessee</t>
+          <t>Peak NAV</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tushar Agrawal</t>
+          <t>Activity Statement / synthesized peak = max(start, end) only. Obtain PortfolioAnalyst for true peak A2.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Account</t>
+          <t>Assessee</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U16595399 — Interactive Brokers LLC (Advisor Client; Advisor: MATCAP WEALTH ADVISORS PRIVATE LIMITED)</t>
+          <t>Tushar Agrawal</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Customer type</t>
+          <t>Account</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>U16595399 — Interactive Brokers LLC (Advisor Client; Advisor: MATCAP WEALTH ADVISORS PRIVATE LIMITED)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Base currency</t>
+          <t>Customer type</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Individual</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Account funded</t>
+          <t>Base currency</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>First deposit n/a (inception statement)</t>
+          <t>USD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Schedule FA period</t>
+          <t>Account funded</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Calendar Year 2025 (01-Jan-2025 to 31-Dec-2025) — for ITR AY 2026-27</t>
+          <t>First deposit n/a (inception statement)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Income / CG period</t>
+          <t>Schedule FA period</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FY 2025-26 (01-Apr-2025 to 31-Mar-2026); also FY 2024-25 sheet for prior year</t>
+          <t>Calendar Year 2025 (01-Jan-2025 to 31-Dec-2025) — for ITR AY 2026-27</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Source data</t>
+          <t>Income / CG period</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IBKR Activity Statements: Inception FY2024-25 + Annual CY2025 + Fiscal FY2025-26</t>
+          <t>FY 2025-26 (01-Apr-2025 to 31-Mar-2026); also FY 2024-25 sheet for prior year</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FIFO method</t>
+          <t>Source data</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Actual buy dates &amp; IBKR Basis from inception replay; splits (LRCX 10:1, NFLX 10:1) applied</t>
+          <t>IBKR Activity Statements: Inception FY2024-25 + Annual CY2025 + Fiscal FY2025-26</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CG reconciliation</t>
+          <t>FIFO method</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sheets 'Capital Gains FY2025-26' / 'FY2024-25' are formula-driven — yellow cells editable; Gain = Sale INR − Comm INR − Cost INR</t>
+          <t>Actual buy dates &amp; IBKR Basis from inception replay; splits (LRCX 10:1, NFLX 10:1) applied</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FX Lookup</t>
+          <t>CG reconciliation</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Editable SBI TT USD/INR &amp; EUR/INR month-end rates + FCY→USD cross rates</t>
+          <t>Sheets 'Capital Gains FY2025-26' / 'FY2024-25' are formula-driven — yellow cells editable; Gain = Sale INR − Comm INR − Cost INR</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Starting NAV CY2025</t>
+          <t>FX Lookup</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>USD 47,669.34</t>
+          <t>Editable SBI TT USD/INR &amp; EUR/INR month-end rates + FCY→USD cross rates</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ending NAV CY2025</t>
+          <t>Starting NAV CY2025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>USD 46,388.40</t>
+          <t>USD 47,669.34</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deposits CY2025</t>
+          <t>Ending NAV CY2025</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>USD 0.00</t>
+          <t>USD 46,388.40</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deposits since inception (to 31-Mar-2025)</t>
+          <t>Deposits CY2025</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3162,79 +3596,79 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dividends CY2025</t>
+          <t>Deposits since inception (to 31-Mar-2025)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>USD 594.18 / INR 51,413 (Rule 115)</t>
+          <t>USD 0.00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Interest CY2025</t>
+          <t>Dividends CY2025</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>USD 82.25 / INR 7,208 (Rule 115)</t>
+          <t>USD 594.18 / INR 51,413 (Rule 115)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dividends FY2025-26</t>
+          <t>Interest CY2025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>USD 829.39 / INR 72,522</t>
+          <t>USD 82.25 / INR 7,208 (Rule 115)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Interest FY2025-26</t>
+          <t>Dividends FY2025-26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>USD 85.97 / INR 7,541</t>
+          <t>USD 829.39 / INR 72,522</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>STCG FY2025-26 (INR)</t>
+          <t>Interest FY2025-26</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>239,329</t>
+          <t>USD 85.97 / INR 7,541</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LTCG FY2025-26 (INR)</t>
+          <t>STCG FY2025-26 (INR)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>239,329</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>STCG FY2024-25 (INR)</t>
+          <t>LTCG FY2025-26 (INR)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3246,7 +3680,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LTCG FY2024-25 (INR)</t>
+          <t>STCG FY2024-25 (INR)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3258,133 +3692,2201 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>A1 Foreign Bank/Depository</t>
+          <t>LTCG FY2024-25 (INR)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Generally N/A separately — multi-currency cash sits inside IBKR custodial account (A2)</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>A2 Custodial Account</t>
+          <t>A1 Foreign Bank/Depository</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Applicable — see sheet; opening: on or before 2024-12-31 (positions held at FY2025-26 start)</t>
+          <t>Generally N/A separately — multi-currency cash sits inside IBKR custodial account (A2)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>A3 Equity &amp; Debt Interest</t>
+          <t>A2 Custodial Account</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Applicable — 58 FIFO lot lines (one row per acquisition lot; sold lots match Capital Gains)</t>
+          <t>Applicable — see sheet; opening: on or before 2024-12-31 (positions held at FY2025-26 start)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>A3 Col C (Name of entity)</t>
+          <t>A3 Equity &amp; Debt Interest</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Symbol only (e.g. NOVd, AAPL). Legal name / address remain in Address &amp; Nature columns.</t>
+          <t>Applicable — 58 FIFO lot lines (one row per acquisition lot; sold lots match Capital Gains)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>A3 vs CG</t>
+          <t>A3 Col C (Name of entity)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sold lots: A3 Initial = CG Cost (INR), A3 Sale = CG Sale (INR), same Rule 115/EUR FX. Multiple buys (e.g. NOVd 21-Mar &amp; 21-Aug) appear as separate A3 rows.</t>
+          <t>Symbol only (e.g. NOVd, AAPL). Legal name / address remain in Address &amp; Nature columns.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ADR country practice</t>
+          <t>A3 vs CG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Underlying issuer country used for ADRs/GDRs (ASML NL, BTI UK, TSM TW, BYDDY CN, HYU KR, RIO UK)</t>
+          <t>Sold lots: A3 Initial = CG Cost (INR), A3 Sale = CG Sale (INR), same Rule 115/EUR FX. Multiple buys (e.g. NOVd 21-Mar &amp; 21-Aug) appear as separate A3 rows.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CPNG</t>
+          <t>ADR country practice</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>USA (Delaware corporation, NYSE) despite Korea operations</t>
+          <t>Underlying issuer country used for ADRs/GDRs (ASML NL, BTI UK, TSM TW, BYDDY CN, HYU KR, RIO UK)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NFLX split</t>
+          <t>CPNG</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10-for-1 split on 14/17-Nov-2025 reflected in FIFO</t>
+          <t>USA (Delaware corporation, NYSE) despite Korea operations</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LRCX split</t>
+          <t>NFLX split</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10-for-1 split on 02/03-Oct-2024 reflected in FIFO (bought 1 pre-split → 10)</t>
+          <t>10-for-1 split on 14/17-Nov-2025 reflected in FIFO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HYU</t>
+          <t>LRCX split</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cash merger acquisition Jul-2025 — sale proceeds USD 1,339.02 reported as redemption proceeds</t>
+          <t>10-for-1 split on 02/03-Oct-2024 reflected in FIFO (bought 1 pre-split → 10)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>HYU</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Cash merger acquisition Jul-2025 — sale proceeds USD 1,339.02 reported as redemption proceeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>Action required</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>1) Confirm exact SBI TT Buy card rates; 2) Obtain PortfolioAnalyst for true peak NAV; 3) Map withholding to Schedule FSI/TR under DTAA.</t>
         </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FY 2026-27 YTD (01-Apr-2026 to 03-Sep-2026) — partial statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Dividends FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>USD 278.11 / INR 26,320</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Interest FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>USD 0.94 / INR 88</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>STCG FY2026-27 YTD (INR)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>896,971</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LTCG FY2026-27 YTD (INR)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>FY2026-27 coverage</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Activity Statement ends 03-Sep-2026 — not full FY. Obtain statement to 31-Mar-2027 for complete year.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Capital gains — FY 2026-27 YTD (01-Apr-2026 to 03-Sep-2026). Partial year — statement ends 03-Sep-2026. FIFO. Yellow cells editable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RECONCILIATION SHEET (formula-driven). Edit yellow cells — P&amp;L recalculates. Gain/(Loss) INR = Sale INR − Comm INR − Cost INR. Holding days &gt;730 → LTCG else STCG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F=E-D | G=IF(F&gt;730,"LTCG","STCG") | L=H*K | M=I*K | Q=L*N (Sale INR) | R=J*P (Comm INR) | S=M*O (Cost INR) | T=Q-R-S (Gain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>CCY</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Acquisition Date</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Sale Date</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Holding Days</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Sale Proceeds (FCY)</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Cost Basis (FCY)</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Comm (USD)</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>FCY→USD Rate</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>Sale Proceeds (USD)</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>Cost (USD)</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>Sale FX Rate</t>
+        </is>
+      </c>
+      <c r="O4" s="1" t="inlineStr">
+        <is>
+          <t>Cost FX Rate</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
+        <is>
+          <t>Comm USD/INR Rate</t>
+        </is>
+      </c>
+      <c r="Q4" s="1" t="inlineStr">
+        <is>
+          <t>Sale (INR)</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>Comm (INR)</t>
+        </is>
+      </c>
+      <c r="S4" s="1" t="inlineStr">
+        <is>
+          <t>Cost (INR)</t>
+        </is>
+      </c>
+      <c r="T4" s="1" t="inlineStr">
+        <is>
+          <t>Gain/(Loss) INR</t>
+        </is>
+      </c>
+      <c r="U4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TIP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="F5">
+        <f>E5-D5</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>IF(F5&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>6209.58</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>6185.5</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <f>H5*K5</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>I5*K5</f>
+        <v/>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q5">
+        <f>L5*N5</f>
+        <v/>
+      </c>
+      <c r="R5">
+        <f>J5*P5</f>
+        <v/>
+      </c>
+      <c r="S5">
+        <f>M5*O5</f>
+        <v/>
+      </c>
+      <c r="T5">
+        <f>Q5-R5-S5</f>
+        <v/>
+      </c>
+      <c r="U5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>URA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>46002</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="F6">
+        <f>E6-D6</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>IF(F6&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>2339.5</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>2374</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <f>H6*K6</f>
+        <v/>
+      </c>
+      <c r="M6">
+        <f>I6*K6</f>
+        <v/>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>88.95</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q6">
+        <f>L6*N6</f>
+        <v/>
+      </c>
+      <c r="R6">
+        <f>J6*P6</f>
+        <v/>
+      </c>
+      <c r="S6">
+        <f>M6*O6</f>
+        <v/>
+      </c>
+      <c r="T6">
+        <f>Q6-R6-S6</f>
+        <v/>
+      </c>
+      <c r="U6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F7">
+        <f>E7-D7</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>IF(F7&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>1134.72</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>1145.07</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <f>H7*K7</f>
+        <v/>
+      </c>
+      <c r="M7">
+        <f>I7*K7</f>
+        <v/>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q7">
+        <f>L7*N7</f>
+        <v/>
+      </c>
+      <c r="R7">
+        <f>J7*P7</f>
+        <v/>
+      </c>
+      <c r="S7">
+        <f>M7*O7</f>
+        <v/>
+      </c>
+      <c r="T7">
+        <f>Q7-R7-S7</f>
+        <v/>
+      </c>
+      <c r="U7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IWR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F8">
+        <f>E8-D8</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IF(F8&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>540.85</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>474.88</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <f>H8*K8</f>
+        <v/>
+      </c>
+      <c r="M8">
+        <f>I8*K8</f>
+        <v/>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q8">
+        <f>L8*N8</f>
+        <v/>
+      </c>
+      <c r="R8">
+        <f>J8*P8</f>
+        <v/>
+      </c>
+      <c r="S8">
+        <f>M8*O8</f>
+        <v/>
+      </c>
+      <c r="T8">
+        <f>Q8-R8-S8</f>
+        <v/>
+      </c>
+      <c r="U8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F9">
+        <f>E9-D9</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IF(F9&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>1435.42</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>1151.67</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <f>H9*K9</f>
+        <v/>
+      </c>
+      <c r="M9">
+        <f>I9*K9</f>
+        <v/>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q9">
+        <f>L9*N9</f>
+        <v/>
+      </c>
+      <c r="R9">
+        <f>J9*P9</f>
+        <v/>
+      </c>
+      <c r="S9">
+        <f>M9*O9</f>
+        <v/>
+      </c>
+      <c r="T9">
+        <f>Q9-R9-S9</f>
+        <v/>
+      </c>
+      <c r="U9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VTV</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F10">
+        <f>E10-D10</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>IF(F10&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>872</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>726.38</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <f>H10*K10</f>
+        <v/>
+      </c>
+      <c r="M10">
+        <f>I10*K10</f>
+        <v/>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q10">
+        <f>L10*N10</f>
+        <v/>
+      </c>
+      <c r="R10">
+        <f>J10*P10</f>
+        <v/>
+      </c>
+      <c r="S10">
+        <f>M10*O10</f>
+        <v/>
+      </c>
+      <c r="T10">
+        <f>Q10-R10-S10</f>
+        <v/>
+      </c>
+      <c r="U10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4568.T</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F11">
+        <f>E11-D11</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>IF(F11&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>254900</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>372297.6</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>203.92</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>0.0063827</v>
+      </c>
+      <c r="L11">
+        <f>H11*K11</f>
+        <v/>
+      </c>
+      <c r="M11">
+        <f>I11*K11</f>
+        <v/>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q11">
+        <f>L11*N11</f>
+        <v/>
+      </c>
+      <c r="R11">
+        <f>J11*P11</f>
+        <v/>
+      </c>
+      <c r="S11">
+        <f>M11*O11</f>
+        <v/>
+      </c>
+      <c r="T11">
+        <f>Q11-R11-S11</f>
+        <v/>
+      </c>
+      <c r="U11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1919</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F12">
+        <f>E12-D12</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>IF(F12&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>6640</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>7206.2</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>25.19</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.12849</v>
+      </c>
+      <c r="L12">
+        <f>H12*K12</f>
+        <v/>
+      </c>
+      <c r="M12">
+        <f>I12*K12</f>
+        <v/>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q12">
+        <f>L12*N12</f>
+        <v/>
+      </c>
+      <c r="R12">
+        <f>J12*P12</f>
+        <v/>
+      </c>
+      <c r="S12">
+        <f>M12*O12</f>
+        <v/>
+      </c>
+      <c r="T12">
+        <f>Q12-R12-S12</f>
+        <v/>
+      </c>
+      <c r="U12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="F13">
+        <f>E13-D13</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>IF(F13&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>2451.51</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>614.53</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <f>H13*K13</f>
+        <v/>
+      </c>
+      <c r="M13">
+        <f>I13*K13</f>
+        <v/>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P13" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q13">
+        <f>L13*N13</f>
+        <v/>
+      </c>
+      <c r="R13">
+        <f>J13*P13</f>
+        <v/>
+      </c>
+      <c r="S13">
+        <f>M13*O13</f>
+        <v/>
+      </c>
+      <c r="T13">
+        <f>Q13-R13-S13</f>
+        <v/>
+      </c>
+      <c r="U13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="F14">
+        <f>E14-D14</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>IF(F14&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>1402.56</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>1203.9</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <f>H14*K14</f>
+        <v/>
+      </c>
+      <c r="M14">
+        <f>I14*K14</f>
+        <v/>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q14">
+        <f>L14*N14</f>
+        <v/>
+      </c>
+      <c r="R14">
+        <f>J14*P14</f>
+        <v/>
+      </c>
+      <c r="S14">
+        <f>M14*O14</f>
+        <v/>
+      </c>
+      <c r="T14">
+        <f>Q14-R14-S14</f>
+        <v/>
+      </c>
+      <c r="U14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AAXJ</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="F15">
+        <f>E15-D15</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>IF(F15&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>482.48</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>346.3</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <f>H15*K15</f>
+        <v/>
+      </c>
+      <c r="M15">
+        <f>I15*K15</f>
+        <v/>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Q15">
+        <f>L15*N15</f>
+        <v/>
+      </c>
+      <c r="R15">
+        <f>J15*P15</f>
+        <v/>
+      </c>
+      <c r="S15">
+        <f>M15*O15</f>
+        <v/>
+      </c>
+      <c r="T15">
+        <f>Q15-R15-S15</f>
+        <v/>
+      </c>
+      <c r="U15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BNO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>33</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>46120</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="F16">
+        <f>E16-D16</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>IF(F16&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>1762.53</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>1507.12</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <f>H16*K16</f>
+        <v/>
+      </c>
+      <c r="M16">
+        <f>I16*K16</f>
+        <v/>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>93.15000000000001</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="Q16">
+        <f>L16*N16</f>
+        <v/>
+      </c>
+      <c r="R16">
+        <f>J16*P16</f>
+        <v/>
+      </c>
+      <c r="S16">
+        <f>M16*O16</f>
+        <v/>
+      </c>
+      <c r="T16">
+        <f>Q16-R16-S16</f>
+        <v/>
+      </c>
+      <c r="U16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SLV</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>159</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>45657</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="F17">
+        <f>E17-D17</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>IF(F17&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>9986.790000000001</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>4524.6</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <f>H17*K17</f>
+        <v/>
+      </c>
+      <c r="M17">
+        <f>I17*K17</f>
+        <v/>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="Q17">
+        <f>L17*N17</f>
+        <v/>
+      </c>
+      <c r="R17">
+        <f>J17*P17</f>
+        <v/>
+      </c>
+      <c r="S17">
+        <f>M17*O17</f>
+        <v/>
+      </c>
+      <c r="T17">
+        <f>Q17-R17-S17</f>
+        <v/>
+      </c>
+      <c r="U17" t="inlineStr"/>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL STCG (INR)</t>
+        </is>
+      </c>
+      <c r="T19" s="4">
+        <f>SUMIF(G5:G17,"STCG",T5:T17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL LTCG (INR)</t>
+        </is>
+      </c>
+      <c r="T20" s="4">
+        <f>SUMIF(G5:G17,"LTCG",T5:T17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL CG (INR)</t>
+        </is>
+      </c>
+      <c r="T21" s="4">
+        <f>T19+T20</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A3:U3"/>
+    <mergeCell ref="A2:U2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Interest &amp; Dividend income — FY 2026-27 YTD (01-Apr-2026 to 03-Sep-2026). Partial — full year needs statement through 31-Mar-2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Amount (FCY)</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Amount (USD)</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>USD/INR (Rule 115)</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Amount (INR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>— INTEREST —</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>USD Credit Interest for Jun-2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="G4" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TOTAL INTEREST</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>— DIVIDENDS —</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NOVO B(DK0062498333) Cash Dividend DKK 3.75 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>150</v>
+      </c>
+      <c r="E8" t="n">
+        <v>23.589</v>
+      </c>
+      <c r="F8" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ASML(NL0010273215) Cash Dividend EUR 2.70 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.3428</v>
+      </c>
+      <c r="F9" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ASML(NL0010273215) Cash Dividend EUR 1.88 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.4165</v>
+      </c>
+      <c r="F10" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1919(CNE1000002J7) Cash Dividend HKD 0.50414 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>252.07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>32.3885</v>
+      </c>
+      <c r="F11" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3064</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4568.T(JP3475350009) Cash Dividend JPY 39 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3900</v>
+      </c>
+      <c r="E12" t="n">
+        <v>24.8925</v>
+      </c>
+      <c r="F12" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2355</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IEF(US4642874402) Cash Dividend USD 0.317166 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F13" t="n">
+        <v>93.15000000000001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IEF(US4642874402) Cash Dividend USD 0.312472 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F14" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TIP(US4642871762) Cash Dividend USD 0.560849 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>31.97</v>
+      </c>
+      <c r="E15" t="n">
+        <v>31.97</v>
+      </c>
+      <c r="F15" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3031</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AAPL(US0378331005) Cash Dividend USD 0.27 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F16" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>WFC(US9497461015) Cash Dividend USD 0.45 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F17" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IEF(US4642874402) Cash Dividend USD 0.317197 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F18" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G18" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TIP(US4642871762) Cash Dividend USD 1.277516 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>72.81999999999999</v>
+      </c>
+      <c r="E19" t="n">
+        <v>72.81999999999999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6889</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>GOOG(US02079K1079) Cash Dividend USD 0.22 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="F20" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G20" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>AAXJ(US4642881829) Cash Dividend USD 0.420785 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F21" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G21" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ICLN(US4642882249) Cash Dividend USD 0.056063 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F22" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G22" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IWR(US4642874998) Cash Dividend USD 0.289405 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F23" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G23" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>VT(US9220427424) Cash Dividend USD 0.5627 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="F24" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G24" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>META(US30303M1027) Cash Dividend USD 0.525 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F25" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G25" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DXJ(US97717W8516) Cash Dividend USD 1.155 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="E26" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="F26" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1093</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BOTZ(US37954Y7159) Cash Dividend USD 0.017986 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F27" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="G27" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>COPX(US37954Y8306) Cash Dividend USD 0.257976 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="E28" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="F28" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>QQQ(US46090E1038) Cash Dividend USD 0.81349 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F29" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="G29" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>JPM(US46625H1005) Cash Dividend USD 1.50 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E30" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F30" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="G30" t="n">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>AAPL(US0378331005) Cash Dividend USD 0.27 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F31" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="G31" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>WFC(US9497461015) Cash Dividend USD 0.50 per Share (Ordinary Dividend)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>12</v>
+      </c>
+      <c r="E32" t="n">
+        <v>12</v>
+      </c>
+      <c r="F32" t="n">
+        <v>95</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TOTAL DIVIDENDS</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>278.11</v>
+      </c>
+      <c r="G33" t="n">
+        <v>26320</v>
       </c>
     </row>
   </sheetData>
@@ -3484,7 +5986,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="n">
         <v>1</v>
@@ -3542,7 +6043,6 @@
           <t>Xiaomi Corporation, Cayman Islands / Beijing ops</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Listed Foreign Equity Share (Company)</t>
@@ -3588,7 +6088,6 @@
           <t>Xiaomi Corporation, Cayman Islands / Beijing ops</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Listed Foreign Equity Share (Company)</t>
@@ -3634,7 +6133,6 @@
           <t>COSCO SHIPPING Holdings Co Ltd, Shanghai</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Listed Foreign Equity Share (Company)</t>
@@ -5375,8 +7873,6 @@
           <t>NOV</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>Listed Foreign Equity / ETF</t>
@@ -6403,7 +8899,6 @@
         <v>112865</v>
       </c>
     </row>
-    <row r="63"/>
     <row r="64">
       <c r="G64" t="inlineStr">
         <is>
@@ -9532,7 +12027,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -9681,7 +12175,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -9830,7 +12323,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -9899,7 +12391,6 @@
         <v>58621</v>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -10218,7 +12709,6 @@
         <v>7208</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -11919,7 +14409,6 @@
         <v>7541</v>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -13733,7 +16222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -18945,6 +21434,806 @@
       </c>
       <c r="H163" t="n">
         <v>-98</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>NOVO B(DK0062498333) Cash Dividend DKK 3.75 per Share - DK Tax</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>-40.5</v>
+      </c>
+      <c r="F164" t="n">
+        <v>-6.369</v>
+      </c>
+      <c r="G164" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="H164" t="n">
+        <v>-606</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="n">
+        <v>46147</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>ASML(NL0010273215) Cash Dividend EUR 2.70 per Share - NL Tax</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="F165" t="n">
+        <v>-0.9514</v>
+      </c>
+      <c r="G165" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="H165" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>ASML(NL0010273215) Cash Dividend EUR 1.88 per Share - NL Tax</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="F166" t="n">
+        <v>-0.6578000000000001</v>
+      </c>
+      <c r="G166" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="H166" t="n">
+        <v>-63</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>1919(CNE1000002J7) Cash Dividend HKD 0.50414 per Share - CN Tax</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>-25.21</v>
+      </c>
+      <c r="F167" t="n">
+        <v>-3.2392</v>
+      </c>
+      <c r="G167" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H167" t="n">
+        <v>-306</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>4568.T(JP3475350009) Cash Dividend JPY 39 per Share - JP Tax</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>-597</v>
+      </c>
+      <c r="F168" t="n">
+        <v>-3.8105</v>
+      </c>
+      <c r="G168" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H168" t="n">
+        <v>-360</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>IEF(US4642874402) Cash Dividend USD 0.317166 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="F169" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="G169" t="n">
+        <v>93.15000000000001</v>
+      </c>
+      <c r="H169" t="n">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>IEF(US4642874402) Cash Dividend USD 0.312472 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="F170" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="G170" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="H170" t="n">
+        <v>-89</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>TIP(US4642871762) Cash Dividend USD 0.560849 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>-7.99</v>
+      </c>
+      <c r="F171" t="n">
+        <v>-7.99</v>
+      </c>
+      <c r="G171" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="H171" t="n">
+        <v>-757</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="n">
+        <v>46156</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>AAPL(US0378331005) Cash Dividend USD 0.27 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F172" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="G172" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="H172" t="n">
+        <v>-32</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>WFC(US9497461015) Cash Dividend USD 0.45 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="F173" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="G173" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H173" t="n">
+        <v>-255</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>IEF(US4642874402) Cash Dividend USD 0.317197 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="F174" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="G174" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H174" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>TIP(US4642871762) Cash Dividend USD 1.277516 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>-18.21</v>
+      </c>
+      <c r="F175" t="n">
+        <v>-18.21</v>
+      </c>
+      <c r="G175" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H175" t="n">
+        <v>-1723</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>GOOG(US02079K1079) Cash Dividend USD 0.22 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="F176" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="G176" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H176" t="n">
+        <v>-16</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>AAXJ(US4642881829) Cash Dividend USD 0.420785 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="F177" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="G177" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H177" t="n">
+        <v>-40</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>ICLN(US4642882249) Cash Dividend USD 0.056063 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="F178" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="G178" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H178" t="n">
+        <v>-26</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>IWR(US4642874998) Cash Dividend USD 0.289405 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="F179" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="G179" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H179" t="n">
+        <v>-34</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>VT(US9220427424) Cash Dividend USD 0.5627 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="F180" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="G180" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H180" t="n">
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>META(US30303M1027) Cash Dividend USD 0.525 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="F181" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="G181" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H181" t="n">
+        <v>-25</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>DXJ(US97717W8516) Cash Dividend USD 1.155 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>-2.89</v>
+      </c>
+      <c r="F182" t="n">
+        <v>-2.89</v>
+      </c>
+      <c r="G182" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="H182" t="n">
+        <v>-273</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>BOTZ(US37954Y7159) Cash Dividend USD 0.017986 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="F183" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="G183" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="H183" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>COPX(US37954Y8306) Cash Dividend USD 0.257976 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>-3.23</v>
+      </c>
+      <c r="F184" t="n">
+        <v>-3.23</v>
+      </c>
+      <c r="G184" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="H184" t="n">
+        <v>-303</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>QQQ(US46090E1038) Cash Dividend USD 0.81349 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="F185" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="G185" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="H185" t="n">
+        <v>-39</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>JPM(US46625H1005) Cash Dividend USD 1.50 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="F186" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="G186" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="H186" t="n">
+        <v>-177</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>AAPL(US0378331005) Cash Dividend USD 0.27 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F187" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="G187" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="H187" t="n">
+        <v>-32</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>WFC(US9497461015) Cash Dividend USD 0.50 per Share - US Tax</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F188" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G188" t="n">
+        <v>95</v>
+      </c>
+      <c r="H188" t="n">
+        <v>-285</v>
       </c>
     </row>
   </sheetData>
@@ -19185,7 +22474,6 @@
         <f>Q5-R5-S5</f>
         <v/>
       </c>
-      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -19260,7 +22548,6 @@
         <f>Q6-R6-S6</f>
         <v/>
       </c>
-      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -19335,7 +22622,6 @@
         <f>Q7-R7-S7</f>
         <v/>
       </c>
-      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19410,7 +22696,6 @@
         <f>Q8-R8-S8</f>
         <v/>
       </c>
-      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -19485,7 +22770,6 @@
         <f>Q9-R9-S9</f>
         <v/>
       </c>
-      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -19560,7 +22844,6 @@
         <f>Q10-R10-S10</f>
         <v/>
       </c>
-      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -19635,7 +22918,6 @@
         <f>Q11-R11-S11</f>
         <v/>
       </c>
-      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19710,7 +22992,6 @@
         <f>Q12-R12-S12</f>
         <v/>
       </c>
-      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19785,7 +23066,6 @@
         <f>Q13-R13-S13</f>
         <v/>
       </c>
-      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19860,7 +23140,6 @@
         <f>Q14-R14-S14</f>
         <v/>
       </c>
-      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -19935,7 +23214,6 @@
         <f>Q15-R15-S15</f>
         <v/>
       </c>
-      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -20010,7 +23288,6 @@
         <f>Q16-R16-S16</f>
         <v/>
       </c>
-      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -20085,7 +23362,6 @@
         <f>Q17-R17-S17</f>
         <v/>
       </c>
-      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -20160,7 +23436,6 @@
         <f>Q18-R18-S18</f>
         <v/>
       </c>
-      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -20235,7 +23510,6 @@
         <f>Q19-R19-S19</f>
         <v/>
       </c>
-      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -20310,7 +23584,6 @@
         <f>Q20-R20-S20</f>
         <v/>
       </c>
-      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -20385,7 +23658,6 @@
         <f>Q21-R21-S21</f>
         <v/>
       </c>
-      <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -20460,7 +23732,6 @@
         <f>Q22-R22-S22</f>
         <v/>
       </c>
-      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -20535,7 +23806,6 @@
         <f>Q23-R23-S23</f>
         <v/>
       </c>
-      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -20610,7 +23880,6 @@
         <f>Q24-R24-S24</f>
         <v/>
       </c>
-      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -20685,7 +23954,6 @@
         <f>Q25-R25-S25</f>
         <v/>
       </c>
-      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -20760,7 +24028,6 @@
         <f>Q26-R26-S26</f>
         <v/>
       </c>
-      <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -21388,7 +24655,6 @@
         <f>Q34-R34-S34</f>
         <v/>
       </c>
-      <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -21463,7 +24729,6 @@
         <f>Q35-R35-S35</f>
         <v/>
       </c>
-      <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -21538,7 +24803,6 @@
         <f>Q36-R36-S36</f>
         <v/>
       </c>
-      <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -21613,9 +24877,7 @@
         <f>Q37-R37-S37</f>
         <v/>
       </c>
-      <c r="U37" t="inlineStr"/>
-    </row>
-    <row r="38"/>
+    </row>
     <row r="39">
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -21649,7 +24911,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>

</xml_diff>